<commit_message>
loading ajax for county_integration_assessment form
</commit_message>
<xml_diff>
--- a/integrations/county_integrations questions.xlsx
+++ b/integrations/county_integrations questions.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\transition-tracker\transitions\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\transition-tracker\integrations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C286937D-3D66-4686-8EDE-A8E325E730D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9850802E-779D-4681-93C3-9B49A2611B76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BA098E8F-21B1-4D71-BE01-2C75F2861913}"/>
   </bookViews>
@@ -1662,299 +1662,299 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="4"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="4"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2295,7 +2295,7 @@
   <cols>
     <col min="1" max="2" width="9.109375" style="4"/>
     <col min="3" max="3" width="29.5546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="8.44140625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="10.21875" style="2" customWidth="1"/>
     <col min="5" max="5" width="100.44140625" style="1" customWidth="1"/>
     <col min="6" max="6" width="94" style="3" customWidth="1"/>
     <col min="7" max="16384" width="9.109375" style="4"/>
@@ -2317,960 +2317,960 @@
       </c>
     </row>
     <row r="5" spans="3:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="94" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="10">
+      <c r="D5" s="9">
         <v>1</v>
       </c>
-      <c r="E5" s="11" t="s">
+      <c r="E5" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="F5" s="12" t="s">
+      <c r="F5" s="11" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="6" spans="3:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C6" s="13"/>
-      <c r="D6" s="14" t="s">
+      <c r="C6" s="95"/>
+      <c r="D6" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="E6" s="15" t="s">
+      <c r="E6" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="F6" s="16" t="s">
+      <c r="F6" s="14" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="7" spans="3:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C7" s="17"/>
-      <c r="D7" s="18" t="s">
+      <c r="C7" s="96"/>
+      <c r="D7" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="E7" s="19" t="s">
+      <c r="E7" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="F7" s="20" t="s">
+      <c r="F7" s="17" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="3:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="C8" s="21" t="s">
+    <row r="8" spans="3:6" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C8" s="83" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="10">
+      <c r="D8" s="9">
         <v>3</v>
       </c>
-      <c r="E8" s="22" t="s">
+      <c r="E8" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="F8" s="12" t="s">
+      <c r="F8" s="11" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="3:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C9" s="23"/>
-      <c r="D9" s="24">
+    <row r="9" spans="3:6" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C9" s="85"/>
+      <c r="D9" s="19">
         <v>4</v>
       </c>
-      <c r="E9" s="25" t="s">
+      <c r="E9" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="F9" s="26" t="s">
+      <c r="F9" s="21" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="10" spans="3:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C10" s="27" t="s">
+      <c r="C10" s="97" t="s">
         <v>18</v>
       </c>
-      <c r="D10" s="10">
+      <c r="D10" s="9">
         <v>5</v>
       </c>
-      <c r="E10" s="28" t="s">
+      <c r="E10" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="F10" s="29" t="s">
+      <c r="F10" s="23" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="11" spans="3:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C11" s="30"/>
-      <c r="D11" s="31">
+      <c r="C11" s="98"/>
+      <c r="D11" s="24">
         <v>6</v>
       </c>
-      <c r="E11" s="32" t="s">
+      <c r="E11" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="F11" s="33" t="s">
+      <c r="F11" s="26" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="12" spans="3:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="C12" s="30"/>
-      <c r="D12" s="10">
+      <c r="C12" s="98"/>
+      <c r="D12" s="9">
         <v>7</v>
       </c>
-      <c r="E12" s="34" t="s">
+      <c r="E12" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="F12" s="35" t="s">
+      <c r="F12" s="28" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="13" spans="3:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="C13" s="30"/>
-      <c r="D13" s="31">
+      <c r="C13" s="98"/>
+      <c r="D13" s="24">
         <v>8</v>
       </c>
-      <c r="E13" s="32" t="s">
+      <c r="E13" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="F13" s="33" t="s">
+      <c r="F13" s="26" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="14" spans="3:6" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C14" s="36"/>
-      <c r="D14" s="31">
+      <c r="C14" s="99"/>
+      <c r="D14" s="24">
         <v>9</v>
       </c>
-      <c r="E14" s="32" t="s">
+      <c r="E14" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="F14" s="33" t="s">
+      <c r="F14" s="26" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="15" spans="3:6" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C15" s="37" t="s">
+      <c r="C15" s="100" t="s">
         <v>29</v>
       </c>
-      <c r="D15" s="10">
+      <c r="D15" s="9">
         <v>10</v>
       </c>
-      <c r="E15" s="38" t="s">
+      <c r="E15" s="29" t="s">
         <v>30</v>
       </c>
-      <c r="F15" s="39" t="s">
+      <c r="F15" s="30" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="16" spans="3:6" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C16" s="37"/>
-      <c r="D16" s="10">
+      <c r="C16" s="100"/>
+      <c r="D16" s="9">
         <v>11</v>
       </c>
-      <c r="E16" s="40" t="s">
+      <c r="E16" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="F16" s="41" t="s">
+      <c r="F16" s="32" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="17" spans="3:9" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C17" s="37"/>
-      <c r="D17" s="10">
+      <c r="C17" s="100"/>
+      <c r="D17" s="9">
         <v>12</v>
       </c>
-      <c r="E17" s="42" t="s">
+      <c r="E17" s="33" t="s">
         <v>34</v>
       </c>
-      <c r="F17" s="43" t="s">
+      <c r="F17" s="34" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="18" spans="3:9" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C18" s="37"/>
-      <c r="D18" s="10">
+      <c r="C18" s="100"/>
+      <c r="D18" s="9">
         <v>13</v>
       </c>
-      <c r="E18" s="42" t="s">
+      <c r="E18" s="33" t="s">
         <v>36</v>
       </c>
-      <c r="F18" s="43" t="s">
+      <c r="F18" s="34" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="19" spans="3:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C19" s="37"/>
-      <c r="D19" s="10">
+      <c r="C19" s="100"/>
+      <c r="D19" s="9">
         <v>14</v>
       </c>
-      <c r="E19" s="44" t="s">
+      <c r="E19" s="35" t="s">
         <v>38</v>
       </c>
-      <c r="F19" s="43" t="s">
+      <c r="F19" s="34" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="20" spans="3:9" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C20" s="37"/>
-      <c r="D20" s="10">
+      <c r="C20" s="100"/>
+      <c r="D20" s="9">
         <v>15</v>
       </c>
-      <c r="E20" s="44" t="s">
+      <c r="E20" s="35" t="s">
         <v>40</v>
       </c>
-      <c r="F20" s="43" t="s">
+      <c r="F20" s="34" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="21" spans="3:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C21" s="37"/>
-      <c r="D21" s="10">
+      <c r="C21" s="100"/>
+      <c r="D21" s="9">
         <v>16</v>
       </c>
-      <c r="E21" s="44" t="s">
+      <c r="E21" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="F21" s="43" t="s">
+      <c r="F21" s="34" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="22" spans="3:9" ht="125.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C22" s="37"/>
-      <c r="D22" s="10">
+      <c r="C22" s="100"/>
+      <c r="D22" s="9">
         <v>17</v>
       </c>
-      <c r="E22" s="45" t="s">
+      <c r="E22" s="36" t="s">
         <v>44</v>
       </c>
-      <c r="F22" s="43" t="s">
+      <c r="F22" s="34" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="23" spans="3:9" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C23" s="37"/>
-      <c r="D23" s="10">
+      <c r="C23" s="100"/>
+      <c r="D23" s="9">
         <v>18</v>
       </c>
-      <c r="E23" s="44" t="s">
+      <c r="E23" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="F23" s="43" t="s">
+      <c r="F23" s="34" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="24" spans="3:9" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C24" s="37"/>
-      <c r="D24" s="10">
+      <c r="C24" s="100"/>
+      <c r="D24" s="9">
         <v>19</v>
       </c>
-      <c r="E24" s="42" t="s">
+      <c r="E24" s="33" t="s">
         <v>47</v>
       </c>
-      <c r="F24" s="43" t="s">
+      <c r="F24" s="34" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="25" spans="3:9" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C25" s="37"/>
-      <c r="D25" s="10">
+      <c r="C25" s="100"/>
+      <c r="D25" s="9">
         <v>20</v>
       </c>
-      <c r="E25" s="44" t="s">
+      <c r="E25" s="35" t="s">
         <v>48</v>
       </c>
-      <c r="F25" s="43" t="s">
+      <c r="F25" s="34" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="26" spans="3:9" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C26" s="37"/>
-      <c r="D26" s="10">
+      <c r="C26" s="100"/>
+      <c r="D26" s="9">
         <v>21</v>
       </c>
-      <c r="E26" s="44" t="s">
+      <c r="E26" s="35" t="s">
         <v>50</v>
       </c>
-      <c r="F26" s="43" t="s">
+      <c r="F26" s="34" t="s">
         <v>51</v>
       </c>
-      <c r="H26" s="46"/>
-      <c r="I26" s="46"/>
+      <c r="H26" s="37"/>
+      <c r="I26" s="37"/>
     </row>
     <row r="27" spans="3:9" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C27" s="47"/>
-      <c r="D27" s="10">
+      <c r="C27" s="101"/>
+      <c r="D27" s="9">
         <v>22</v>
       </c>
-      <c r="E27" s="48" t="s">
+      <c r="E27" s="38" t="s">
         <v>52</v>
       </c>
-      <c r="F27" s="49" t="s">
+      <c r="F27" s="39" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="28" spans="3:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C28" s="50" t="s">
+      <c r="C28" s="102" t="s">
         <v>54</v>
       </c>
-      <c r="D28" s="10">
+      <c r="D28" s="9">
         <v>23</v>
       </c>
-      <c r="E28" s="51" t="s">
+      <c r="E28" s="40" t="s">
         <v>55</v>
       </c>
-      <c r="F28" s="52" t="s">
+      <c r="F28" s="41" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="29" spans="3:9" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C29" s="53"/>
-      <c r="D29" s="10">
+      <c r="C29" s="103"/>
+      <c r="D29" s="9">
         <v>24</v>
       </c>
-      <c r="E29" s="54" t="s">
+      <c r="E29" s="42" t="s">
         <v>57</v>
       </c>
-      <c r="F29" s="55" t="s">
+      <c r="F29" s="43" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="30" spans="3:9" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C30" s="56" t="s">
+      <c r="C30" s="104" t="s">
         <v>59</v>
       </c>
-      <c r="D30" s="10">
+      <c r="D30" s="9">
         <v>25</v>
       </c>
-      <c r="E30" s="51" t="s">
+      <c r="E30" s="40" t="s">
         <v>60</v>
       </c>
-      <c r="F30" s="57" t="s">
+      <c r="F30" s="44" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="31" spans="3:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C31" s="58"/>
-      <c r="D31" s="10">
+      <c r="C31" s="105"/>
+      <c r="D31" s="9">
         <v>26</v>
       </c>
-      <c r="E31" s="59" t="s">
+      <c r="E31" s="45" t="s">
         <v>62</v>
       </c>
-      <c r="F31" s="43" t="s">
+      <c r="F31" s="34" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="32" spans="3:9" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C32" s="58"/>
-      <c r="D32" s="10">
+      <c r="C32" s="105"/>
+      <c r="D32" s="9">
         <v>27</v>
       </c>
-      <c r="E32" s="59" t="s">
+      <c r="E32" s="45" t="s">
         <v>64</v>
       </c>
-      <c r="F32" s="43" t="s">
+      <c r="F32" s="34" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="33" spans="3:6" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C33" s="58"/>
-      <c r="D33" s="10">
+      <c r="C33" s="105"/>
+      <c r="D33" s="9">
         <v>28</v>
       </c>
-      <c r="E33" s="59" t="s">
+      <c r="E33" s="45" t="s">
         <v>66</v>
       </c>
-      <c r="F33" s="43" t="s">
+      <c r="F33" s="34" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="34" spans="3:6" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C34" s="58"/>
-      <c r="D34" s="10">
+      <c r="C34" s="105"/>
+      <c r="D34" s="9">
         <v>29</v>
       </c>
-      <c r="E34" s="59" t="s">
+      <c r="E34" s="45" t="s">
         <v>68</v>
       </c>
-      <c r="F34" s="43" t="s">
+      <c r="F34" s="34" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="35" spans="3:6" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C35" s="58"/>
-      <c r="D35" s="10">
+      <c r="C35" s="105"/>
+      <c r="D35" s="9">
         <v>30</v>
       </c>
-      <c r="E35" s="59" t="s">
+      <c r="E35" s="45" t="s">
         <v>70</v>
       </c>
-      <c r="F35" s="43" t="s">
+      <c r="F35" s="34" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="36" spans="3:6" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C36" s="60"/>
-      <c r="D36" s="10">
+      <c r="C36" s="106"/>
+      <c r="D36" s="9">
         <v>31</v>
       </c>
-      <c r="E36" s="54" t="s">
+      <c r="E36" s="42" t="s">
         <v>72</v>
       </c>
-      <c r="F36" s="39" t="s">
+      <c r="F36" s="30" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="37" spans="3:6" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C37" s="61" t="s">
+      <c r="C37" s="80" t="s">
         <v>74</v>
       </c>
-      <c r="D37" s="10">
+      <c r="D37" s="9">
         <v>32</v>
       </c>
-      <c r="E37" s="62" t="s">
+      <c r="E37" s="46" t="s">
         <v>75</v>
       </c>
-      <c r="F37" s="63" t="s">
+      <c r="F37" s="47" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="38" spans="3:6" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C38" s="64"/>
-      <c r="D38" s="10">
+      <c r="C38" s="81"/>
+      <c r="D38" s="9">
         <v>33</v>
       </c>
-      <c r="E38" s="65" t="s">
+      <c r="E38" s="48" t="s">
         <v>77</v>
       </c>
-      <c r="F38" s="66" t="s">
+      <c r="F38" s="49" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="39" spans="3:6" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C39" s="64"/>
-      <c r="D39" s="10">
+      <c r="C39" s="81"/>
+      <c r="D39" s="9">
         <v>34</v>
       </c>
-      <c r="E39" s="65" t="s">
+      <c r="E39" s="48" t="s">
         <v>79</v>
       </c>
-      <c r="F39" s="66" t="s">
+      <c r="F39" s="49" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="40" spans="3:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C40" s="64"/>
-      <c r="D40" s="10">
+      <c r="C40" s="81"/>
+      <c r="D40" s="9">
         <v>35</v>
       </c>
-      <c r="E40" s="65" t="s">
+      <c r="E40" s="48" t="s">
         <v>81</v>
       </c>
-      <c r="F40" s="66" t="s">
+      <c r="F40" s="49" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="41" spans="3:6" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C41" s="64"/>
-      <c r="D41" s="10">
+      <c r="C41" s="81"/>
+      <c r="D41" s="9">
         <v>36</v>
       </c>
-      <c r="E41" s="65" t="s">
+      <c r="E41" s="48" t="s">
         <v>83</v>
       </c>
-      <c r="F41" s="66" t="s">
+      <c r="F41" s="49" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="42" spans="3:6" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C42" s="64"/>
-      <c r="D42" s="10">
+      <c r="C42" s="81"/>
+      <c r="D42" s="9">
         <v>37</v>
       </c>
-      <c r="E42" s="65" t="s">
+      <c r="E42" s="48" t="s">
         <v>85</v>
       </c>
-      <c r="F42" s="66" t="s">
+      <c r="F42" s="49" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="43" spans="3:6" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C43" s="64"/>
-      <c r="D43" s="10">
+      <c r="C43" s="81"/>
+      <c r="D43" s="9">
         <v>38</v>
       </c>
-      <c r="E43" s="67" t="s">
+      <c r="E43" s="50" t="s">
         <v>87</v>
       </c>
-      <c r="F43" s="26" t="s">
+      <c r="F43" s="21" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="44" spans="3:6" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C44" s="64"/>
-      <c r="D44" s="10">
+      <c r="C44" s="81"/>
+      <c r="D44" s="9">
         <v>39</v>
       </c>
-      <c r="E44" s="67" t="s">
+      <c r="E44" s="50" t="s">
         <v>89</v>
       </c>
-      <c r="F44" s="26" t="s">
+      <c r="F44" s="21" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="45" spans="3:6" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C45" s="64"/>
-      <c r="D45" s="10">
+      <c r="C45" s="81"/>
+      <c r="D45" s="9">
         <v>40</v>
       </c>
-      <c r="E45" s="68" t="s">
+      <c r="E45" s="51" t="s">
         <v>91</v>
       </c>
-      <c r="F45" s="69" t="s">
+      <c r="F45" s="52" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="46" spans="3:6" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C46" s="70"/>
-      <c r="D46" s="10">
+      <c r="C46" s="82"/>
+      <c r="D46" s="9">
         <v>41</v>
       </c>
-      <c r="E46" s="68" t="s">
+      <c r="E46" s="51" t="s">
         <v>93</v>
       </c>
-      <c r="F46" s="69" t="s">
+      <c r="F46" s="52" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="47" spans="3:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C47" s="21" t="s">
+      <c r="C47" s="83" t="s">
         <v>95</v>
       </c>
-      <c r="D47" s="10">
+      <c r="D47" s="9">
         <v>42</v>
       </c>
-      <c r="E47" s="71" t="s">
+      <c r="E47" s="53" t="s">
         <v>96</v>
       </c>
-      <c r="F47" s="12" t="s">
+      <c r="F47" s="11" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="48" spans="3:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C48" s="72"/>
-      <c r="D48" s="10">
+      <c r="C48" s="84"/>
+      <c r="D48" s="9">
         <v>43</v>
       </c>
-      <c r="E48" s="65" t="s">
+      <c r="E48" s="48" t="s">
         <v>98</v>
       </c>
-      <c r="F48" s="66" t="s">
+      <c r="F48" s="49" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="49" spans="3:6" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C49" s="72"/>
-      <c r="D49" s="10">
+      <c r="C49" s="84"/>
+      <c r="D49" s="9">
         <v>44</v>
       </c>
-      <c r="E49" s="65" t="s">
+      <c r="E49" s="48" t="s">
         <v>100</v>
       </c>
-      <c r="F49" s="66" t="s">
+      <c r="F49" s="49" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="50" spans="3:6" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C50" s="72"/>
-      <c r="D50" s="10">
+      <c r="C50" s="84"/>
+      <c r="D50" s="9">
         <v>45</v>
       </c>
-      <c r="E50" s="65" t="s">
+      <c r="E50" s="48" t="s">
         <v>102</v>
       </c>
-      <c r="F50" s="66" t="s">
+      <c r="F50" s="49" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="51" spans="3:6" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C51" s="72"/>
-      <c r="D51" s="10">
+      <c r="C51" s="84"/>
+      <c r="D51" s="9">
         <v>46</v>
       </c>
-      <c r="E51" s="65" t="s">
+      <c r="E51" s="48" t="s">
         <v>104</v>
       </c>
-      <c r="F51" s="66" t="s">
+      <c r="F51" s="49" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="52" spans="3:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C52" s="72"/>
-      <c r="D52" s="10">
+      <c r="C52" s="84"/>
+      <c r="D52" s="9">
         <v>47</v>
       </c>
-      <c r="E52" s="65" t="s">
+      <c r="E52" s="48" t="s">
         <v>106</v>
       </c>
-      <c r="F52" s="66" t="s">
+      <c r="F52" s="49" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="53" spans="3:6" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C53" s="23"/>
-      <c r="D53" s="10">
+      <c r="C53" s="85"/>
+      <c r="D53" s="9">
         <v>48</v>
       </c>
-      <c r="E53" s="67" t="s">
+      <c r="E53" s="50" t="s">
         <v>108</v>
       </c>
-      <c r="F53" s="26" t="s">
+      <c r="F53" s="21" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="54" spans="3:6" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C54" s="23"/>
-      <c r="D54" s="10">
+      <c r="C54" s="85"/>
+      <c r="D54" s="9">
         <v>49</v>
       </c>
-      <c r="E54" s="67" t="s">
+      <c r="E54" s="50" t="s">
         <v>110</v>
       </c>
-      <c r="F54" s="26" t="s">
+      <c r="F54" s="21" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="55" spans="3:6" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C55" s="73"/>
-      <c r="D55" s="10">
+      <c r="C55" s="86"/>
+      <c r="D55" s="9">
         <v>50</v>
       </c>
-      <c r="E55" s="74" t="s">
+      <c r="E55" s="54" t="s">
         <v>112</v>
       </c>
-      <c r="F55" s="20" t="s">
+      <c r="F55" s="17" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="56" spans="3:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C56" s="75" t="s">
+      <c r="C56" s="87" t="s">
         <v>114</v>
       </c>
-      <c r="D56" s="10">
+      <c r="D56" s="9">
         <v>51</v>
       </c>
-      <c r="E56" s="71" t="s">
+      <c r="E56" s="53" t="s">
         <v>115</v>
       </c>
-      <c r="F56" s="12" t="s">
+      <c r="F56" s="11" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="57" spans="3:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C57" s="76"/>
-      <c r="D57" s="10">
+      <c r="C57" s="88"/>
+      <c r="D57" s="9">
         <v>52</v>
       </c>
-      <c r="E57" s="65" t="s">
+      <c r="E57" s="48" t="s">
         <v>117</v>
       </c>
-      <c r="F57" s="66" t="s">
+      <c r="F57" s="49" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="58" spans="3:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C58" s="76"/>
-      <c r="D58" s="10">
+      <c r="C58" s="88"/>
+      <c r="D58" s="9">
         <v>53</v>
       </c>
-      <c r="E58" s="65" t="s">
+      <c r="E58" s="48" t="s">
         <v>119</v>
       </c>
-      <c r="F58" s="66" t="s">
+      <c r="F58" s="49" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="59" spans="3:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C59" s="76"/>
-      <c r="D59" s="10">
+      <c r="C59" s="88"/>
+      <c r="D59" s="9">
         <v>54</v>
       </c>
-      <c r="E59" s="65" t="s">
+      <c r="E59" s="48" t="s">
         <v>121</v>
       </c>
-      <c r="F59" s="66" t="s">
+      <c r="F59" s="49" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="60" spans="3:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C60" s="76"/>
-      <c r="D60" s="10">
+      <c r="C60" s="88"/>
+      <c r="D60" s="9">
         <v>55</v>
       </c>
-      <c r="E60" s="65" t="s">
+      <c r="E60" s="48" t="s">
         <v>123</v>
       </c>
-      <c r="F60" s="66" t="s">
+      <c r="F60" s="49" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="61" spans="3:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C61" s="76"/>
-      <c r="D61" s="10">
+      <c r="C61" s="88"/>
+      <c r="D61" s="9">
         <v>56</v>
       </c>
-      <c r="E61" s="65" t="s">
+      <c r="E61" s="48" t="s">
         <v>125</v>
       </c>
-      <c r="F61" s="66" t="s">
+      <c r="F61" s="49" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="62" spans="3:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C62" s="76"/>
-      <c r="D62" s="10">
+      <c r="C62" s="88"/>
+      <c r="D62" s="9">
         <v>57</v>
       </c>
-      <c r="E62" s="65" t="s">
+      <c r="E62" s="48" t="s">
         <v>127</v>
       </c>
-      <c r="F62" s="66" t="s">
+      <c r="F62" s="49" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="63" spans="3:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C63" s="76"/>
-      <c r="D63" s="10">
+      <c r="C63" s="88"/>
+      <c r="D63" s="9">
         <v>58</v>
       </c>
-      <c r="E63" s="74" t="s">
+      <c r="E63" s="54" t="s">
         <v>129</v>
       </c>
-      <c r="F63" s="20" t="s">
+      <c r="F63" s="17" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="64" spans="3:6" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C64" s="76"/>
-      <c r="D64" s="10">
+      <c r="C64" s="88"/>
+      <c r="D64" s="9">
         <v>59</v>
       </c>
-      <c r="E64" s="65" t="s">
+      <c r="E64" s="48" t="s">
         <v>131</v>
       </c>
-      <c r="F64" s="66" t="s">
+      <c r="F64" s="49" t="s">
         <v>132</v>
       </c>
     </row>
     <row r="65" spans="3:6" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C65" s="77"/>
-      <c r="D65" s="10">
+      <c r="C65" s="89"/>
+      <c r="D65" s="9">
         <v>60</v>
       </c>
-      <c r="E65" s="65" t="s">
+      <c r="E65" s="48" t="s">
         <v>133</v>
       </c>
-      <c r="F65" s="66" t="s">
+      <c r="F65" s="49" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="66" spans="3:6" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C66" s="78" t="s">
+      <c r="C66" s="90" t="s">
         <v>135</v>
       </c>
-      <c r="D66" s="10">
+      <c r="D66" s="9">
         <v>61</v>
       </c>
-      <c r="E66" s="62" t="s">
+      <c r="E66" s="46" t="s">
         <v>136</v>
       </c>
-      <c r="F66" s="63" t="s">
+      <c r="F66" s="47" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="67" spans="3:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C67" s="79"/>
-      <c r="D67" s="10">
+      <c r="C67" s="91"/>
+      <c r="D67" s="9">
         <v>62</v>
       </c>
-      <c r="E67" s="80" t="s">
+      <c r="E67" s="55" t="s">
         <v>138</v>
       </c>
-      <c r="F67" s="20" t="s">
+      <c r="F67" s="17" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="68" spans="3:6" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C68" s="81" t="s">
+      <c r="C68" s="92" t="s">
         <v>140</v>
       </c>
-      <c r="D68" s="10">
+      <c r="D68" s="9">
         <v>63</v>
       </c>
-      <c r="E68" s="82" t="s">
+      <c r="E68" s="56" t="s">
         <v>141</v>
       </c>
-      <c r="F68" s="66" t="s">
+      <c r="F68" s="49" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="69" spans="3:6" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C69" s="83"/>
-      <c r="D69" s="10">
+      <c r="C69" s="93"/>
+      <c r="D69" s="9">
         <v>64</v>
       </c>
-      <c r="E69" s="67" t="s">
+      <c r="E69" s="50" t="s">
         <v>143</v>
       </c>
-      <c r="F69" s="26" t="s">
+      <c r="F69" s="21" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="70" spans="3:6" ht="102" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C70" s="84" t="s">
+      <c r="C70" s="57" t="s">
         <v>145</v>
       </c>
-      <c r="D70" s="10">
+      <c r="D70" s="9">
         <v>65</v>
       </c>
-      <c r="E70" s="85" t="s">
+      <c r="E70" s="58" t="s">
         <v>146</v>
       </c>
-      <c r="F70" s="86" t="s">
+      <c r="F70" s="59" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="71" spans="3:6" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C71" s="87" t="s">
+      <c r="C71" s="76" t="s">
         <v>148</v>
       </c>
-      <c r="D71" s="10">
+      <c r="D71" s="9">
         <v>66</v>
       </c>
-      <c r="E71" s="88" t="s">
+      <c r="E71" s="60" t="s">
         <v>149</v>
       </c>
-      <c r="F71" s="89" t="s">
+      <c r="F71" s="61" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="72" spans="3:6" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C72" s="87"/>
-      <c r="D72" s="10">
+      <c r="C72" s="76"/>
+      <c r="D72" s="9">
         <v>67</v>
       </c>
-      <c r="E72" s="90" t="s">
+      <c r="E72" s="62" t="s">
         <v>151</v>
       </c>
-      <c r="F72" s="91" t="s">
+      <c r="F72" s="63" t="s">
         <v>152</v>
       </c>
     </row>
     <row r="73" spans="3:6" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C73" s="92" t="s">
+      <c r="C73" s="75" t="s">
         <v>153</v>
       </c>
-      <c r="D73" s="10">
+      <c r="D73" s="9">
         <v>68</v>
       </c>
-      <c r="E73" s="88" t="s">
+      <c r="E73" s="60" t="s">
         <v>154</v>
       </c>
-      <c r="F73" s="89" t="s">
+      <c r="F73" s="61" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="74" spans="3:6" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C74" s="92"/>
-      <c r="D74" s="10">
+      <c r="C74" s="75"/>
+      <c r="D74" s="9">
         <v>69</v>
       </c>
-      <c r="E74" s="90" t="s">
+      <c r="E74" s="62" t="s">
         <v>156</v>
       </c>
-      <c r="F74" s="93" t="s">
+      <c r="F74" s="64" t="s">
         <v>157</v>
       </c>
     </row>
     <row r="75" spans="3:6" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C75" s="87" t="s">
+      <c r="C75" s="76" t="s">
         <v>158</v>
       </c>
-      <c r="D75" s="10">
+      <c r="D75" s="9">
         <v>70</v>
       </c>
-      <c r="E75" s="88" t="s">
+      <c r="E75" s="60" t="s">
         <v>159</v>
       </c>
-      <c r="F75" s="94" t="s">
+      <c r="F75" s="65" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="76" spans="3:6" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C76" s="87"/>
-      <c r="D76" s="10">
+      <c r="C76" s="76"/>
+      <c r="D76" s="9">
         <v>71</v>
       </c>
-      <c r="E76" s="95" t="s">
+      <c r="E76" s="66" t="s">
         <v>161</v>
       </c>
-      <c r="F76" s="69" t="s">
+      <c r="F76" s="52" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="77" spans="3:6" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C77" s="87"/>
-      <c r="D77" s="10">
+      <c r="C77" s="76"/>
+      <c r="D77" s="9">
         <v>72</v>
       </c>
-      <c r="E77" s="95" t="s">
+      <c r="E77" s="66" t="s">
         <v>163</v>
       </c>
-      <c r="F77" s="69" t="s">
+      <c r="F77" s="52" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="78" spans="3:6" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C78" s="87"/>
-      <c r="D78" s="96">
+      <c r="C78" s="76"/>
+      <c r="D78" s="67">
         <v>73</v>
       </c>
-      <c r="E78" s="90" t="s">
+      <c r="E78" s="62" t="s">
         <v>165</v>
       </c>
-      <c r="F78" s="93" t="s">
+      <c r="F78" s="64" t="s">
         <v>166</v>
       </c>
     </row>
     <row r="79" spans="3:6" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C79" s="97" t="s">
+      <c r="C79" s="77" t="s">
         <v>167</v>
       </c>
-      <c r="D79" s="10">
+      <c r="D79" s="9">
         <v>74</v>
       </c>
-      <c r="E79" s="90" t="s">
+      <c r="E79" s="62" t="s">
         <v>168</v>
       </c>
-      <c r="F79" s="93" t="s">
+      <c r="F79" s="64" t="s">
         <v>169</v>
       </c>
     </row>
     <row r="80" spans="3:6" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C80" s="98"/>
-      <c r="D80" s="96">
+      <c r="C80" s="78"/>
+      <c r="D80" s="67">
         <v>75</v>
       </c>
-      <c r="E80" s="90" t="s">
+      <c r="E80" s="62" t="s">
         <v>170</v>
       </c>
-      <c r="F80" s="93" t="s">
+      <c r="F80" s="64" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="81" spans="3:6" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C81" s="99"/>
-      <c r="D81" s="96">
+      <c r="C81" s="79"/>
+      <c r="D81" s="67">
         <v>76</v>
       </c>
-      <c r="E81" s="90" t="s">
+      <c r="E81" s="62" t="s">
         <v>172</v>
       </c>
-      <c r="F81" s="93" t="s">
+      <c r="F81" s="64" t="s">
         <v>173</v>
       </c>
     </row>
@@ -3278,51 +3278,57 @@
       <c r="D82" s="1"/>
     </row>
     <row r="84" spans="3:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E84" s="100" t="s">
+      <c r="E84" s="68" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="85" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="E85" s="101"/>
+      <c r="E85" s="69"/>
     </row>
     <row r="86" spans="3:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="E86" s="102" t="s">
+      <c r="E86" s="70" t="s">
         <v>175</v>
       </c>
     </row>
     <row r="87" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="E87" s="103"/>
+      <c r="E87" s="71"/>
     </row>
     <row r="88" spans="3:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="E88" s="102" t="s">
+      <c r="E88" s="70" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="89" spans="3:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="E89" s="104" t="s">
+      <c r="E89" s="72" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="90" spans="3:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="E90" s="104" t="s">
+      <c r="E90" s="72" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="91" spans="3:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E91" s="105"/>
+      <c r="E91" s="73"/>
     </row>
     <row r="95" spans="3:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E95" s="100" t="s">
+      <c r="E95" s="68" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="96" spans="3:6" ht="63" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E96" s="106" t="s">
+      <c r="E96" s="74" t="s">
         <v>180</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="C30:C36"/>
+    <mergeCell ref="C5:C7"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="C10:C14"/>
+    <mergeCell ref="C15:C27"/>
+    <mergeCell ref="C28:C29"/>
     <mergeCell ref="C73:C74"/>
     <mergeCell ref="C75:C78"/>
     <mergeCell ref="C79:C81"/>
@@ -3332,12 +3338,6 @@
     <mergeCell ref="C66:C67"/>
     <mergeCell ref="C68:C69"/>
     <mergeCell ref="C71:C72"/>
-    <mergeCell ref="C5:C7"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="C10:C14"/>
-    <mergeCell ref="C15:C27"/>
-    <mergeCell ref="C28:C29"/>
-    <mergeCell ref="C30:C36"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>